<commit_message>
update sửa lỗi nhập file
</commit_message>
<xml_diff>
--- a/wwwroot/template/TemPlateQuote.xlsx
+++ b/wwwroot/template/TemPlateQuote.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\khanhmf\Cost Managerment\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D24112-D211-467D-AC3A-8F6AF1A67275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28921A7A-4735-4D7B-902D-FD1C66E91630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F4BD22E2-5202-4BAA-B608-770E176E4E09}"/>
   </bookViews>
@@ -3579,13 +3579,34 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3607,24 +3628,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3634,18 +3646,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4123,18 +4123,18 @@
     </row>
     <row r="4" spans="1:32" ht="11.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="C4" s="49"/>
-      <c r="D4" s="50"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="39"/>
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
-      <c r="H4" s="49" t="s">
+      <c r="H4" s="38" t="s">
         <v>214</v>
       </c>
-      <c r="I4" s="51"/>
+      <c r="I4" s="40"/>
       <c r="J4" s="9"/>
       <c r="K4" s="25"/>
       <c r="M4" s="9"/>
@@ -4156,14 +4156,14 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="50"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="39"/>
       <c r="E5" s="25"/>
       <c r="F5" s="25"/>
       <c r="G5" s="25"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="51"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="40"/>
       <c r="J5" s="25"/>
       <c r="K5" s="25"/>
       <c r="L5" s="18"/>
@@ -4187,17 +4187,17 @@
       <c r="AD5" s="9"/>
     </row>
     <row r="6" spans="1:32" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="43" t="s">
         <v>264</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
       <c r="J6" s="18"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
@@ -4257,15 +4257,15 @@
       <c r="L7" s="26">
         <v>12</v>
       </c>
-      <c r="M7" s="41">
+      <c r="M7" s="48">
         <f>L7+1</f>
         <v>13</v>
       </c>
-      <c r="N7" s="42"/>
-      <c r="O7" s="42"/>
-      <c r="P7" s="42"/>
-      <c r="Q7" s="42"/>
-      <c r="R7" s="43"/>
+      <c r="N7" s="49"/>
+      <c r="O7" s="49"/>
+      <c r="P7" s="49"/>
+      <c r="Q7" s="49"/>
+      <c r="R7" s="50"/>
       <c r="S7" s="24">
         <v>14</v>
       </c>
@@ -4323,106 +4323,106 @@
       </c>
     </row>
     <row r="8" spans="1:32" s="7" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="41" t="s">
         <v>215</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="41" t="s">
         <v>216</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="E8" s="39" t="s">
+      <c r="E8" s="41" t="s">
         <v>218</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="41" t="s">
         <v>219</v>
       </c>
-      <c r="G8" s="39" t="s">
+      <c r="G8" s="41" t="s">
         <v>220</v>
       </c>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="41" t="s">
         <v>222</v>
       </c>
-      <c r="I8" s="39" t="s">
+      <c r="I8" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="J8" s="39" t="s">
+      <c r="J8" s="41" t="s">
         <v>221</v>
       </c>
-      <c r="K8" s="39" t="s">
+      <c r="K8" s="41" t="s">
         <v>224</v>
       </c>
-      <c r="L8" s="39" t="s">
+      <c r="L8" s="41" t="s">
         <v>225</v>
       </c>
-      <c r="M8" s="44" t="s">
+      <c r="M8" s="51" t="s">
         <v>231</v>
       </c>
-      <c r="N8" s="45"/>
-      <c r="O8" s="45"/>
-      <c r="P8" s="45"/>
-      <c r="Q8" s="45"/>
-      <c r="R8" s="46"/>
-      <c r="S8" s="39" t="s">
+      <c r="N8" s="52"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="52"/>
+      <c r="Q8" s="52"/>
+      <c r="R8" s="53"/>
+      <c r="S8" s="41" t="s">
         <v>235</v>
       </c>
-      <c r="T8" s="39" t="s">
+      <c r="T8" s="41" t="s">
         <v>236</v>
       </c>
-      <c r="U8" s="39" t="s">
+      <c r="U8" s="41" t="s">
         <v>232</v>
       </c>
-      <c r="V8" s="39" t="s">
+      <c r="V8" s="41" t="s">
         <v>233</v>
       </c>
-      <c r="W8" s="39" t="s">
+      <c r="W8" s="41" t="s">
         <v>237</v>
       </c>
-      <c r="X8" s="39" t="s">
+      <c r="X8" s="41" t="s">
         <v>238</v>
       </c>
-      <c r="Y8" s="39" t="s">
+      <c r="Y8" s="41" t="s">
         <v>239</v>
       </c>
-      <c r="Z8" s="39" t="s">
+      <c r="Z8" s="41" t="s">
         <v>240</v>
       </c>
-      <c r="AA8" s="39" t="s">
+      <c r="AA8" s="41" t="s">
         <v>241</v>
       </c>
-      <c r="AB8" s="39" t="s">
+      <c r="AB8" s="41" t="s">
         <v>242</v>
       </c>
-      <c r="AC8" s="39" t="s">
+      <c r="AC8" s="41" t="s">
         <v>243</v>
       </c>
-      <c r="AD8" s="39" t="s">
+      <c r="AD8" s="41" t="s">
         <v>244</v>
       </c>
-      <c r="AE8" s="38" t="s">
+      <c r="AE8" s="47" t="s">
         <v>245</v>
       </c>
-      <c r="AF8" s="38" t="s">
+      <c r="AF8" s="47" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:32" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="48"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
-      <c r="I9" s="40"/>
-      <c r="J9" s="40"/>
-      <c r="K9" s="40"/>
-      <c r="L9" s="40"/>
+      <c r="A9" s="46"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+      <c r="K9" s="42"/>
+      <c r="L9" s="42"/>
       <c r="M9" s="19" t="s">
         <v>226</v>
       </c>
@@ -4441,20 +4441,20 @@
       <c r="R9" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="S9" s="40"/>
-      <c r="T9" s="40"/>
-      <c r="U9" s="40"/>
-      <c r="V9" s="40"/>
-      <c r="W9" s="40"/>
-      <c r="X9" s="40"/>
-      <c r="Y9" s="40"/>
-      <c r="Z9" s="40"/>
-      <c r="AA9" s="40"/>
-      <c r="AB9" s="40"/>
-      <c r="AC9" s="40"/>
-      <c r="AD9" s="40"/>
-      <c r="AE9" s="38"/>
-      <c r="AF9" s="38"/>
+      <c r="S9" s="42"/>
+      <c r="T9" s="42"/>
+      <c r="U9" s="42"/>
+      <c r="V9" s="42"/>
+      <c r="W9" s="42"/>
+      <c r="X9" s="42"/>
+      <c r="Y9" s="42"/>
+      <c r="Z9" s="42"/>
+      <c r="AA9" s="42"/>
+      <c r="AB9" s="42"/>
+      <c r="AC9" s="42"/>
+      <c r="AD9" s="42"/>
+      <c r="AE9" s="47"/>
+      <c r="AF9" s="47"/>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
@@ -29098,23 +29098,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="Y8:Y9"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="U8:U9"/>
-    <mergeCell ref="V8:V9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="X8:X9"/>
     <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="AF8:AF9"/>
@@ -29131,6 +29114,23 @@
     <mergeCell ref="Z8:Z9"/>
     <mergeCell ref="AA8:AA9"/>
     <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="S8:S9"/>
+    <mergeCell ref="A6:I6"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA10:AA569" xr:uid="{A48AEAD6-16A7-419C-9ADE-A3A1D0E68BC1}">
@@ -29193,11 +29193,11 @@
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
       <c r="E2" s="20" t="s">
         <v>209</v>
       </c>
@@ -29207,11 +29207,11 @@
       <c r="G2" s="21"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="56" t="s">
         <v>201</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
       <c r="E3" s="20" t="s">
         <v>209</v>
       </c>
@@ -29226,10 +29226,10 @@
       <c r="B4" s="29">
         <v>1</v>
       </c>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="56"/>
+      <c r="D4" s="60"/>
       <c r="E4" s="20" t="s">
         <v>204</v>
       </c>
@@ -29242,10 +29242,10 @@
       <c r="B5" s="29">
         <v>2</v>
       </c>
-      <c r="C5" s="57" t="s">
+      <c r="C5" s="54" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="58"/>
+      <c r="D5" s="55"/>
       <c r="E5" s="20" t="s">
         <v>204</v>
       </c>
@@ -29257,10 +29257,10 @@
       <c r="B6" s="29">
         <v>3</v>
       </c>
-      <c r="C6" s="57" t="s">
+      <c r="C6" s="54" t="s">
         <v>216</v>
       </c>
-      <c r="D6" s="58"/>
+      <c r="D6" s="55"/>
       <c r="E6" s="20" t="s">
         <v>209</v>
       </c>
@@ -29275,10 +29275,10 @@
       <c r="B7" s="29">
         <v>4</v>
       </c>
-      <c r="C7" s="57" t="s">
+      <c r="C7" s="54" t="s">
         <v>217</v>
       </c>
-      <c r="D7" s="58"/>
+      <c r="D7" s="55"/>
       <c r="E7" s="20" t="s">
         <v>209</v>
       </c>
@@ -29293,10 +29293,10 @@
       <c r="B8" s="29">
         <v>5</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="C8" s="54" t="s">
         <v>218</v>
       </c>
-      <c r="D8" s="58"/>
+      <c r="D8" s="55"/>
       <c r="E8" s="20" t="s">
         <v>206</v>
       </c>
@@ -29311,10 +29311,10 @@
       <c r="B9" s="29">
         <v>6</v>
       </c>
-      <c r="C9" s="57" t="s">
+      <c r="C9" s="54" t="s">
         <v>219</v>
       </c>
-      <c r="D9" s="58"/>
+      <c r="D9" s="55"/>
       <c r="E9" s="20" t="s">
         <v>204</v>
       </c>
@@ -29329,10 +29329,10 @@
       <c r="B10" s="29">
         <v>7</v>
       </c>
-      <c r="C10" s="57" t="s">
+      <c r="C10" s="54" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="58"/>
+      <c r="D10" s="55"/>
       <c r="E10" s="20" t="s">
         <v>209</v>
       </c>
@@ -29347,10 +29347,10 @@
       <c r="B11" s="29">
         <v>8</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="54" t="s">
         <v>222</v>
       </c>
-      <c r="D11" s="58"/>
+      <c r="D11" s="55"/>
       <c r="E11" s="20" t="s">
         <v>209</v>
       </c>
@@ -29365,10 +29365,10 @@
       <c r="B12" s="29">
         <v>9</v>
       </c>
-      <c r="C12" s="57" t="s">
+      <c r="C12" s="54" t="s">
         <v>223</v>
       </c>
-      <c r="D12" s="58"/>
+      <c r="D12" s="55"/>
       <c r="E12" s="20" t="s">
         <v>209</v>
       </c>
@@ -29381,10 +29381,10 @@
       <c r="B13" s="29">
         <v>10</v>
       </c>
-      <c r="C13" s="57" t="s">
+      <c r="C13" s="54" t="s">
         <v>221</v>
       </c>
-      <c r="D13" s="58"/>
+      <c r="D13" s="55"/>
       <c r="E13" s="20" t="s">
         <v>204</v>
       </c>
@@ -29397,10 +29397,10 @@
       <c r="B14" s="29">
         <v>11</v>
       </c>
-      <c r="C14" s="57" t="s">
+      <c r="C14" s="54" t="s">
         <v>224</v>
       </c>
-      <c r="D14" s="58"/>
+      <c r="D14" s="55"/>
       <c r="E14" s="20" t="s">
         <v>204</v>
       </c>
@@ -29413,10 +29413,10 @@
       <c r="B15" s="29">
         <v>12</v>
       </c>
-      <c r="C15" s="57" t="s">
+      <c r="C15" s="54" t="s">
         <v>225</v>
       </c>
-      <c r="D15" s="58"/>
+      <c r="D15" s="55"/>
       <c r="E15" s="20" t="s">
         <v>209</v>
       </c>
@@ -29428,11 +29428,11 @@
       </c>
     </row>
     <row r="16" spans="2:7" ht="72" x14ac:dyDescent="0.25">
-      <c r="B16" s="60">
+      <c r="B16" s="57">
         <f>B15+1</f>
         <v>13</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="58" t="s">
         <v>231</v>
       </c>
       <c r="D16" s="30" t="s">
@@ -29449,8 +29449,8 @@
       </c>
     </row>
     <row r="17" spans="2:7" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="60"/>
-      <c r="C17" s="54"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="58"/>
       <c r="D17" s="30" t="s">
         <v>227</v>
       </c>
@@ -29465,8 +29465,8 @@
       </c>
     </row>
     <row r="18" spans="2:7" ht="72" x14ac:dyDescent="0.25">
-      <c r="B18" s="60"/>
-      <c r="C18" s="54"/>
+      <c r="B18" s="57"/>
+      <c r="C18" s="58"/>
       <c r="D18" s="30" t="s">
         <v>228</v>
       </c>
@@ -29481,8 +29481,8 @@
       </c>
     </row>
     <row r="19" spans="2:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="B19" s="60"/>
-      <c r="C19" s="54"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="58"/>
       <c r="D19" s="30" t="s">
         <v>229</v>
       </c>
@@ -29497,8 +29497,8 @@
       </c>
     </row>
     <row r="20" spans="2:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="B20" s="60"/>
-      <c r="C20" s="54"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="58"/>
       <c r="D20" s="30" t="s">
         <v>230</v>
       </c>
@@ -29513,8 +29513,8 @@
       </c>
     </row>
     <row r="21" spans="2:7" ht="48" x14ac:dyDescent="0.25">
-      <c r="B21" s="60"/>
-      <c r="C21" s="54"/>
+      <c r="B21" s="57"/>
+      <c r="C21" s="58"/>
       <c r="D21" s="30" t="s">
         <v>234</v>
       </c>
@@ -29532,10 +29532,10 @@
       <c r="B22" s="31">
         <v>14</v>
       </c>
-      <c r="C22" s="57" t="s">
+      <c r="C22" s="54" t="s">
         <v>235</v>
       </c>
-      <c r="D22" s="58"/>
+      <c r="D22" s="55"/>
       <c r="E22" s="20" t="s">
         <v>206</v>
       </c>
@@ -29551,10 +29551,10 @@
         <f t="shared" ref="B23:B35" si="0">B22+1</f>
         <v>15</v>
       </c>
-      <c r="C23" s="57" t="s">
+      <c r="C23" s="54" t="s">
         <v>236</v>
       </c>
-      <c r="D23" s="58"/>
+      <c r="D23" s="55"/>
       <c r="E23" s="20" t="s">
         <v>206</v>
       </c>
@@ -29570,10 +29570,10 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C24" s="57" t="s">
+      <c r="C24" s="54" t="s">
         <v>232</v>
       </c>
-      <c r="D24" s="58"/>
+      <c r="D24" s="55"/>
       <c r="E24" s="20" t="s">
         <v>206</v>
       </c>
@@ -29589,10 +29589,10 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C25" s="57" t="s">
+      <c r="C25" s="54" t="s">
         <v>233</v>
       </c>
-      <c r="D25" s="58"/>
+      <c r="D25" s="55"/>
       <c r="E25" s="20" t="s">
         <v>206</v>
       </c>
@@ -29608,10 +29608,10 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C26" s="57" t="s">
+      <c r="C26" s="54" t="s">
         <v>237</v>
       </c>
-      <c r="D26" s="58"/>
+      <c r="D26" s="55"/>
       <c r="E26" s="20" t="s">
         <v>211</v>
       </c>
@@ -29627,10 +29627,10 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C27" s="57" t="s">
+      <c r="C27" s="54" t="s">
         <v>238</v>
       </c>
-      <c r="D27" s="58"/>
+      <c r="D27" s="55"/>
       <c r="E27" s="20" t="s">
         <v>209</v>
       </c>
@@ -29646,10 +29646,10 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C28" s="57" t="s">
+      <c r="C28" s="54" t="s">
         <v>239</v>
       </c>
-      <c r="D28" s="58"/>
+      <c r="D28" s="55"/>
       <c r="E28" s="20" t="s">
         <v>209</v>
       </c>
@@ -29665,10 +29665,10 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C29" s="57" t="s">
+      <c r="C29" s="54" t="s">
         <v>240</v>
       </c>
-      <c r="D29" s="58"/>
+      <c r="D29" s="55"/>
       <c r="E29" s="20" t="s">
         <v>209</v>
       </c>
@@ -29684,10 +29684,10 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C30" s="57" t="s">
+      <c r="C30" s="54" t="s">
         <v>241</v>
       </c>
-      <c r="D30" s="58"/>
+      <c r="D30" s="55"/>
       <c r="E30" s="20" t="s">
         <v>204</v>
       </c>
@@ -29703,10 +29703,10 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C31" s="57" t="s">
+      <c r="C31" s="54" t="s">
         <v>242</v>
       </c>
-      <c r="D31" s="58"/>
+      <c r="D31" s="55"/>
       <c r="E31" s="20" t="s">
         <v>204</v>
       </c>
@@ -29722,10 +29722,10 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C32" s="57" t="s">
+      <c r="C32" s="54" t="s">
         <v>243</v>
       </c>
-      <c r="D32" s="58"/>
+      <c r="D32" s="55"/>
       <c r="E32" s="20" t="s">
         <v>204</v>
       </c>
@@ -29739,10 +29739,10 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C33" s="57" t="s">
+      <c r="C33" s="54" t="s">
         <v>244</v>
       </c>
-      <c r="D33" s="58"/>
+      <c r="D33" s="55"/>
       <c r="E33" s="20" t="s">
         <v>204</v>
       </c>
@@ -29758,10 +29758,10 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C34" s="54" t="s">
+      <c r="C34" s="58" t="s">
         <v>245</v>
       </c>
-      <c r="D34" s="54"/>
+      <c r="D34" s="58"/>
       <c r="E34" s="20" t="s">
         <v>206</v>
       </c>
@@ -29777,10 +29777,10 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C35" s="54" t="s">
+      <c r="C35" s="58" t="s">
         <v>246</v>
       </c>
-      <c r="D35" s="54"/>
+      <c r="D35" s="58"/>
       <c r="E35" s="20" t="s">
         <v>206</v>
       </c>
@@ -29794,20 +29794,6 @@
   </sheetData>
   <autoFilter ref="B1:H35" xr:uid="{9A62EE61-DA4A-4471-B605-47242F0A4DEA}"/>
   <mergeCells count="30">
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="C16:C21"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C4:D4"/>
@@ -29824,6 +29810,20 @@
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="C16:C21"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>